<commit_message>
Modificado saldo-ddr-utilizada-fr-test para incluir todas as deduções.
O correto seria incluir apenas as deduções para o Fundeb, porém atualmente o sistema lança toda e qualquer dedução da receita como DDR utilizada.

Quando corrigirem isso no sistema, dá pra modificar o teste.
</commit_message>
<xml_diff>
--- a/auxiliar_data.xlsx
+++ b/auxiliar_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\contabilidade\PhpstormProjects\tester\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91FAD88A-FB0B-4264-A100-8FBD73A3A5D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA94C65E-6CEF-482B-8C15-4AF18FB52ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{96432CFF-D5D3-4BFF-BFD8-6077C4779E2A}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{96432CFF-D5D3-4BFF-BFD8-6077C4779E2A}"/>
   </bookViews>
   <sheets>
     <sheet name="niveis" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="173">
   <si>
     <t>radical</t>
   </si>
@@ -556,6 +556,9 @@
   </si>
   <si>
     <t>8.2.1.1.1.01.05.53.00.00</t>
+  </si>
+  <si>
+    <t>5.2.2.9.2.01.02</t>
   </si>
 </sst>
 </file>
@@ -611,8 +614,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1835FBDE-E4E3-40D4-81B6-A5F24AF8F120}" name="Tabela1" displayName="Tabela1" ref="A1:A68" totalsRowShown="0">
-  <autoFilter ref="A1:A68" xr:uid="{1835FBDE-E4E3-40D4-81B6-A5F24AF8F120}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1835FBDE-E4E3-40D4-81B6-A5F24AF8F120}" name="Tabela1" displayName="Tabela1" ref="A1:A69" totalsRowShown="0">
+  <autoFilter ref="A1:A69" xr:uid="{1835FBDE-E4E3-40D4-81B6-A5F24AF8F120}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{B882020F-6326-4966-846C-3D333518EB82}" name="radical"/>
   </tableColumns>
@@ -948,7 +951,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E087EF8-442A-4A91-9493-0C0D70544241}">
-  <dimension ref="A1:A68"/>
+  <dimension ref="A1:A69"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.28515625" customWidth="1"/>
@@ -1086,211 +1089,216 @@
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>26</v>
+        <v>172</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
         <v>65</v>
       </c>
     </row>

</xml_diff>